<commit_message>
Add Monthly/Quarterly UX Metrics suite, UAT env support, and RAS hardenings.
Introduce the BI MQ UX Metrics regression pack with POM/probe/Excel, wire portal URLs through config including UAT, and harden Revenue Assurance soft status flows for headed runs.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/Revenue_Assurance_Dashboard_Regression.xlsx
+++ b/docs/Revenue_Assurance_Dashboard_Regression.xlsx
@@ -13,9 +13,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="195">
-  <si>
-    <t>Profile: US / GDC Test Site 2 | Type: Regression (reversible status mutations only) | Total TCs: 34 | Revenue Assurance Dashboard</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="205">
+  <si>
+    <t>Profile: US / GDC Test Site 2 | Type: Regression (reversible status mutations only) | Total TCs: 36 | Revenue Assurance Dashboard</t>
   </si>
   <si>
     <t>SoT = live probe + Help Center Revenue Assurance Product Overview. Suite home: Improve Revenue → Revenue Assurance Dashboard.</t>
@@ -42,24 +42,30 @@
     <t>Business Insights — Improve Revenue</t>
   </si>
   <si>
+    <t>Chrome</t>
+  </si>
+  <si>
+    <t>REG-RAS-003, REG-RAS-004, REG-RAS-005, REG-RAS-006, REG-RAS-007, REG-RAS-035</t>
+  </si>
+  <si>
     <t>Detail</t>
   </si>
   <si>
     <t>REG-RAS-019, REG-RAS-020, REG-RAS-021, REG-RAS-022, REG-RAS-023, REG-RAS-024</t>
   </si>
   <si>
-    <t>Chrome</t>
-  </si>
-  <si>
-    <t>REG-RAS-003, REG-RAS-004, REG-RAS-005, REG-RAS-006, REG-RAS-007</t>
-  </si>
-  <si>
     <t>Cards</t>
   </si>
   <si>
     <t>REG-RAS-013, REG-RAS-014, REG-RAS-015, REG-RAS-016</t>
   </si>
   <si>
+    <t>Table</t>
+  </si>
+  <si>
+    <t>REG-RAS-017, REG-RAS-018, REG-RAS-034</t>
+  </si>
+  <si>
     <t>Hero</t>
   </si>
   <si>
@@ -72,12 +78,6 @@
     <t>REG-RAS-010, REG-RAS-011</t>
   </si>
   <si>
-    <t>Table</t>
-  </si>
-  <si>
-    <t>REG-RAS-017, REG-RAS-018</t>
-  </si>
-  <si>
     <t>Status</t>
   </si>
   <si>
@@ -93,7 +93,7 @@
     <t>Recovery</t>
   </si>
   <si>
-    <t>REG-RAS-032, REG-RAS-034</t>
+    <t>REG-RAS-032, REG-RAS-036</t>
   </si>
   <si>
     <t>Navigation</t>
@@ -141,10 +141,10 @@
     <t>TOTAL</t>
   </si>
   <si>
-    <t>REG-RAS-001 .. REG-RAS-034</t>
-  </si>
-  <si>
-    <t>Execution: Passed (35/35) — Executed 2026-08-25 (headed chromium-regression, workers=1). Soft annotations: Share opened=false; table search fill timeout (recovered); Data Science SOURCE DATA soft-empty; Status New soft-miss (no count mutation); REG-RAS-026 sampled Implemented + Internal Declined (In Progress/Declined soft-skipped to protect serial timeout); card AREAS sum format-tolerant; Declined filter label may show External Declined. Allure: allure_reports/ras-report/index.html</t>
+    <t>REG-RAS-001 .. REG-RAS-036</t>
+  </si>
+  <si>
+    <t>Execution: Passed (37/37) — 2026-08-27 — 37/37 incl. BUG-4870 (REG-RAS-034) + BUG-4848 (REG-RAS-035). Allure: allure_reports/ras-report/index.html</t>
   </si>
   <si>
     <t>Test Case ID</t>
@@ -176,7 +176,7 @@
 2. title Revenue Assurance Dashboard.</t>
   </si>
   <si>
-    <t>Passed (35/35)</t>
+    <t>Passed (37/37)</t>
   </si>
   <si>
     <t>GDC Test Site 2; core inventory settles</t>
@@ -593,6 +593,37 @@
     <t>REG-RAS-034</t>
   </si>
   <si>
+    <t>BUG-4870: All Recommendations table fits viewport (Internal Review; multi-width)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Internal Review Show Me (or hero Show Me)
+2. scroll #revenueAssuranceTable
+3. hard assert 1440px
+4. soft annotate 1280/1100.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. At 1440px table fits wrapper (checkbox + Date not clipped
+2. no horizontal overflow). 1280/1100px annotated soft (BUG-4870 / BTTS-3916).</t>
+  </si>
+  <si>
+    <t>REG-RAS-035</t>
+  </si>
+  <si>
+    <t>BUG-4848: Improve Revenue ($) toolbar tooltip uses portal term</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Read revenue portal term from page config
+2. hover top-toolbar $ / Revenue Assurance icon
+3. inspect title/bootstrap tooltip.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Tooltip reflects configured portal term (not hardcoded "revenue" when term customized)
+2. shows Revenue Assurance / Rev Assure label (BUG-4848 / BTTS-3886).</t>
+  </si>
+  <si>
+    <t>REG-RAS-036</t>
+  </si>
+  <si>
     <t>Restore initial context; suite home healthy</t>
   </si>
   <si>
@@ -615,16 +646,16 @@
     <t>Header style: bold white text on #1F4E79</t>
   </si>
   <si>
-    <t>Total cases: 34 (REG-RAS-001 .. REG-RAS-034)</t>
+    <t>Total cases: 36 (REG-RAS-001 .. REG-RAS-036)</t>
   </si>
   <si>
     <t>Automation: tests/regression_tests/US2/business-insights/improve-revenue/revenue-assurance/revenue.assurance.regression.spec.ts</t>
   </si>
   <si>
-    <t>Execution status: Passed (35/35)</t>
-  </si>
-  <si>
-    <t>Execution note: Executed 2026-08-25 (headed chromium-regression, workers=1). Soft annotations: Share opened=false; table search fill timeout (recovered); Data Science SOURCE DATA soft-empty; Status New soft-miss (no count mutation); REG-RAS-026 sampled Implemented + Internal Declined (In Progress/Declined soft-skipped to protect serial timeout); card AREAS sum format-tolerant; Declined filter label may show External Declined. Allure: allure_reports/ras-report/index.html</t>
+    <t>Execution status: Passed (37/37)</t>
+  </si>
+  <si>
+    <t>Execution note: 2026-08-27 — 37/37 incl. BUG-4870 (REG-RAS-034) + BUG-4848 (REG-RAS-035). Allure: allure_reports/ras-report/index.html</t>
   </si>
   <si>
     <t>Exact home: Business Insights / Improve Revenue / Revenue Assurance (route revenue-assurance/dashboard).</t>
@@ -642,7 +673,13 @@
     <t>Dollar amounts and status counts are live-data — never hard-code.</t>
   </si>
   <si>
-    <t>Stable hosts: #recommendationsChart, #platformChart, #revenueAssuranceTable, #internal-review-records-btn, #recPerfViewDataModal.</t>
+    <t>Stable hosts: #recommendationsChart, #platformChart, #revenueAssuranceTable, #revenueAssuranceTable-table-viewport, #internal-review-records-btn, #recPerfViewDataModal.</t>
+  </si>
+  <si>
+    <t>BUG-4870 (REG-RAS-034): All Recommendations table must fit viewport — checkbox + Date columns not clipped at 1440/1280/1100.</t>
+  </si>
+  <si>
+    <t>BUG-4848 (REG-RAS-035): Top-toolbar $ icon tooltip must honor revenue portal term configuration.</t>
   </si>
   <si>
     <t>npm run test:regression:us2:revenue-assurance</t>
@@ -1135,7 +1172,7 @@
         <v>11</v>
       </c>
       <c r="D6" s="5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>12</v>
@@ -1163,7 +1200,7 @@
         <v>15</v>
       </c>
       <c r="D8" s="5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>16</v>
@@ -1345,7 +1382,7 @@
         <v>7</v>
       </c>
       <c r="D21" s="6">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E21" s="6" t="s">
         <v>42</v>
@@ -1372,7 +1409,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1474,7 +1511,7 @@
         <v>8</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>58</v>
@@ -1500,7 +1537,7 @@
         <v>8</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>62</v>
@@ -1526,7 +1563,7 @@
         <v>8</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>66</v>
@@ -1552,7 +1589,7 @@
         <v>8</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>70</v>
@@ -1578,7 +1615,7 @@
         <v>8</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>74</v>
@@ -1604,7 +1641,7 @@
         <v>8</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>78</v>
@@ -1630,7 +1667,7 @@
         <v>8</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>82</v>
@@ -1656,7 +1693,7 @@
         <v>8</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>86</v>
@@ -1682,7 +1719,7 @@
         <v>8</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>90</v>
@@ -1838,7 +1875,7 @@
         <v>8</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E18" s="5" t="s">
         <v>113</v>
@@ -1864,7 +1901,7 @@
         <v>8</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E19" s="5" t="s">
         <v>117</v>
@@ -1890,7 +1927,7 @@
         <v>8</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E20" s="5" t="s">
         <v>121</v>
@@ -1916,7 +1953,7 @@
         <v>8</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E21" s="5" t="s">
         <v>125</v>
@@ -1942,7 +1979,7 @@
         <v>8</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E22" s="5" t="s">
         <v>129</v>
@@ -1968,7 +2005,7 @@
         <v>8</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E23" s="5" t="s">
         <v>133</v>
@@ -1994,7 +2031,7 @@
         <v>8</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E24" s="5" t="s">
         <v>137</v>
@@ -2020,7 +2057,7 @@
         <v>8</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E25" s="5" t="s">
         <v>141</v>
@@ -2269,7 +2306,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="35" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="35" ht="76" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
         <v>176</v>
       </c>
@@ -2280,7 +2317,7 @@
         <v>8</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="E35" s="5" t="s">
         <v>177</v>
@@ -2289,18 +2326,70 @@
         <v>178</v>
       </c>
       <c r="G35" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="H35" s="5" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="36" ht="60" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="F36" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="G36" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="H36" s="5" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="37" ht="48" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D37" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E37" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="F37" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="G37" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="H35" s="5" t="s">
+      <c r="H37" s="5" t="s">
         <v>53</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" sqref="H10:H35">
+    <dataValidation type="list" allowBlank="1" sqref="H10:H37">
       <formula1>"Not Executed,Pass,Fail,Blocked,Skipped"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="H2:H35">
+    <dataValidation type="list" allowBlank="1" sqref="H2:H37">
       <formula1>"Not Executed,Pass,Fail,Blocked,Skipped"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2311,7 +2400,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
@@ -2319,37 +2408,37 @@
   <sheetData>
     <row r="1" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
@@ -2359,47 +2448,57 @@
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>194</v>
+        <v>202</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>204</v>
       </c>
     </row>
   </sheetData>

</xml_diff>